<commit_message>
Research of UV light
</commit_message>
<xml_diff>
--- a/SLSS V5/SLSS V5 BoM.xlsx
+++ b/SLSS V5/SLSS V5 BoM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\edwar\Documents\SLSS\SLSS V5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C32D7493-F28B-43F1-B345-D5E40B4F8B55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66652A29-18FF-47D8-ADBA-B91CFC8EF113}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{0175BE9B-09DB-4935-9617-04C8C213D07E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="38">
   <si>
     <t>No</t>
   </si>
@@ -126,6 +126,30 @@
   </si>
   <si>
     <t>621-2170</t>
+  </si>
+  <si>
+    <t>https://uk.rs-online.com/web/p/uvc-lamps/2411306</t>
+  </si>
+  <si>
+    <t>241-1306</t>
+  </si>
+  <si>
+    <t>UVC Light</t>
+  </si>
+  <si>
+    <t>germocidal light</t>
+  </si>
+  <si>
+    <t>https://uk.rs-online.com/web/p/heatsinks/1846719</t>
+  </si>
+  <si>
+    <t>30mm heatsink</t>
+  </si>
+  <si>
+    <t>Heatsink</t>
+  </si>
+  <si>
+    <t>184-6719</t>
   </si>
 </sst>
 </file>
@@ -663,10 +687,41 @@
       <c r="B7">
         <v>5</v>
       </c>
-      <c r="F7" s="1"/>
+      <c r="C7" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G7" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="F8" s="1"/>
+      <c r="B8">
+        <v>6</v>
+      </c>
+      <c r="C8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" t="s">
+        <v>35</v>
+      </c>
+      <c r="E8">
+        <v>2</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G8" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.35">
       <c r="F9" s="1"/>
@@ -759,8 +814,9 @@
     <hyperlink ref="F14" r:id="rId1" display="https://docs.arduino.cc/resources/pinouts/ABX00028-full-pinout.pdf" xr:uid="{36804345-AEB4-4E7D-9BC7-C81B0111FE34}"/>
     <hyperlink ref="F15" r:id="rId2" location="technical-details" display="https://www.adafruit.com/product/326 - technical-details" xr:uid="{4DCB4C25-963E-47BD-BBC1-72406EC1CDC3}"/>
     <hyperlink ref="F3" r:id="rId3" xr:uid="{A0A63F22-757F-463A-BAC4-D32816C56DA8}"/>
+    <hyperlink ref="F5" r:id="rId4" xr:uid="{354B0B53-CBFA-4FC4-B068-1AE81EC69D5D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added SMD LED to BoM
</commit_message>
<xml_diff>
--- a/SLSS V5/SLSS V5 BoM.xlsx
+++ b/SLSS V5/SLSS V5 BoM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\edwar\Documents\SLSS\SLSS V5\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://npluk-my.sharepoint.com/personal/james_edwards_npl_co_uk/Documents/Documents/SLSS/SLSS V5/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66652A29-18FF-47D8-ADBA-B91CFC8EF113}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{66652A29-18FF-47D8-ADBA-B91CFC8EF113}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{821009F8-DA0A-4D4F-A682-16306C674B77}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{0175BE9B-09DB-4935-9617-04C8C213D07E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{0175BE9B-09DB-4935-9617-04C8C213D07E}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="42">
   <si>
     <t>No</t>
   </si>
@@ -150,6 +150,18 @@
   </si>
   <si>
     <t>184-6719</t>
+  </si>
+  <si>
+    <t>RGB LED SMD</t>
+  </si>
+  <si>
+    <t>LED</t>
+  </si>
+  <si>
+    <t>Kingbright3.2 V, 4.1 V, 4.5 V RGB LED 5050 SMD, KAAF-5050RGBS-13 | RS</t>
+  </si>
+  <si>
+    <t>872-1724</t>
   </si>
 </sst>
 </file>
@@ -724,7 +736,24 @@
       </c>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="F9" s="1"/>
+      <c r="B9">
+        <v>7</v>
+      </c>
+      <c r="C9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E9">
+        <v>6</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G9" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.35">
       <c r="F10" s="1"/>
@@ -815,8 +844,9 @@
     <hyperlink ref="F15" r:id="rId2" location="technical-details" display="https://www.adafruit.com/product/326 - technical-details" xr:uid="{4DCB4C25-963E-47BD-BBC1-72406EC1CDC3}"/>
     <hyperlink ref="F3" r:id="rId3" xr:uid="{A0A63F22-757F-463A-BAC4-D32816C56DA8}"/>
     <hyperlink ref="F5" r:id="rId4" xr:uid="{354B0B53-CBFA-4FC4-B068-1AE81EC69D5D}"/>
+    <hyperlink ref="F9" r:id="rId5" display="https://uk.rs-online.com/web/p/leds/8721724" xr:uid="{368DA346-24B6-4715-9D7D-22DC54DCFC68}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>
 </worksheet>
 </file>
</xml_diff>